<commit_message>
move files to the appropriate locations
</commit_message>
<xml_diff>
--- a/analyses/data/Metadata_Table_OH_removed.xlsx
+++ b/analyses/data/Metadata_Table_OH_removed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexikeene/Documents/Research/PhD_Research/diverse_collections/github/analyses/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775327A1-9203-7C45-A83F-ED13C58FE29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D52CD61-3B77-B04A-AA13-264E82A6819B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36040" yWindow="-2200" windowWidth="34480" windowHeight="21100" xr2:uid="{2FD151FF-324E-8F4B-B590-25CABDE34919}"/>
+    <workbookView xWindow="-35620" yWindow="1440" windowWidth="34480" windowHeight="21100" xr2:uid="{2FD151FF-324E-8F4B-B590-25CABDE34919}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata_Table" sheetId="1" r:id="rId1"/>
@@ -15592,7 +15592,7 @@
       </c>
       <c r="P137" s="16">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q137" s="1">
         <v>1</v>
@@ -15604,14 +15604,14 @@
         <v>1</v>
       </c>
       <c r="T137" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U137" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V137" s="16">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W137" s="1">
         <v>1</v>
@@ -15623,10 +15623,10 @@
         <v>1</v>
       </c>
       <c r="Z137" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA137" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="AB137" s="1" t="s">
         <v>183</v>

</xml_diff>